<commit_message>
docs: integrate 1000-question benchmark into XLSX and update DOCX manifesto
</commit_message>
<xml_diff>
--- a/docs/SymboLM_Benchmark_Data_and_Math_Evaluation.xlsx
+++ b/docs/SymboLM_Benchmark_Data_and_Math_Evaluation.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="200_Cross_Domain_Benchmark" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Stages_1_to_5_Progress" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Mathematical_Complexity_Models" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="DeepSeek_CoDesign_224x" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Grant_Budget_Allocation" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="200_Cross_Domain_Benchmark" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stages_1_to_5_Progress" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mathematical_Complexity_Models" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DeepSeek_CoDesign_224x" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1000_Multi_Year_Benchmark" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,10 +20,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
-    <numFmt numFmtId="166" formatCode="$#,##0"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -133,7 +132,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -168,11 +167,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1596,19 +1593,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Emergent Ventures &amp; 1517 Fund Grant Budget Allocation ($20,000 – $25,000)</t>
+          <t>SymboLM-1.5B-v1.0 1,000-Question Multi-Year Benchmark (Tesla P100 GPU)</t>
         </is>
       </c>
     </row>
@@ -1616,97 +1615,166 @@
     <row r="3">
       <c r="A3" s="16" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>Benchmark Year</t>
         </is>
       </c>
       <c r="B3" s="16" t="inlineStr">
         <is>
-          <t>Allocation ($ USD)</t>
+          <t>Sample Count</t>
         </is>
       </c>
       <c r="C3" s="16" t="inlineStr">
         <is>
-          <t>Share (%)</t>
+          <t>Pass@1 Accuracy</t>
         </is>
       </c>
       <c r="D3" s="16" t="inlineStr">
         <is>
-          <t>Operational Impact &amp; Milestone Deliverables</t>
+          <t>SymboLM Avg Tokens</t>
+        </is>
+      </c>
+      <c r="E3" s="16" t="inlineStr">
+        <is>
+          <t>Baseline CoT Avg Tokens</t>
+        </is>
+      </c>
+      <c r="F3" s="16" t="inlineStr">
+        <is>
+          <t>Token Savings</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>1. Electrical &amp; Power Resilience (Rupandehi, Nepal)</t>
+          <t>2021 (GSM8K, SVAMP, Arithmetic)</t>
         </is>
       </c>
       <c r="B4" s="18" t="n">
-        <v>5000</v>
+        <v>200</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Pure sine-wave inverter, LiFePO4 battery storage (0ms switchover), and dual-WAN failover router to ensure continuous connection during regional grid blackouts.</t>
-        </is>
+        <v>0.72</v>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>114.3</v>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>198</v>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>0.423</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>2. Dedicated Cloud Compute Clusters</t>
+          <t>2022 (AMC 10/12 Invariants, Vieta)</t>
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>12000</v>
+        <v>200</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.48</v>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>Dedicated A100/H100 GPU clusters (Lambda Labs / RunPod) to scale SymboLM from 1.5B parameters to 14B and 32B foundation models, executing multi-thousand sample GRPO rollouts.</t>
-        </is>
+        <v>0.71</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>128</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>214.5</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>0.403</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>3. Living &amp; Physical Care Runway (12 Months)</t>
+          <t>2023 (MATH Olympiad Derangements)</t>
         </is>
       </c>
       <c r="B6" s="18" t="n">
-        <v>8000</v>
+        <v>200</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>0.32</v>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>12-month domestic and caregiving assistance runway in Rupandehi, Nepal, providing physical autonomy to conduct full-time independent AI research.</t>
-        </is>
+        <v>0.845</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>128</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>264.5</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>0.516</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>TOTAL UNRESTRICTED FELLOWSHIP</t>
-        </is>
-      </c>
-      <c r="B7" s="19">
-        <f>SUM(B4:B6)</f>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>2024 (AIME 2024, Legendre Valuations)</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="n">
+        <v>200</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>0.725</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>128</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>283</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>0.548</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>2026 (Modern Math 2026, Multi-Moduli CRT)</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="n">
+        <v>200</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>128</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>309</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>0.586</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>OVERALL 1,000-QUESTION SUITE</t>
+        </is>
+      </c>
+      <c r="B9" s="12">
+        <f>SUM(B4:B8)</f>
         <v/>
       </c>
-      <c r="C7" s="20">
-        <f>SUM(C4:C6)</f>
-        <v/>
-      </c>
-      <c r="D7" s="12" t="inlineStr">
-        <is>
-          <t>Permanent elimination of power, compute, and physical bottlenecks.</t>
-        </is>
+      <c r="C9" s="13" t="n">
+        <v>0.676</v>
+      </c>
+      <c r="D9" s="12" t="n">
+        <v>125.3</v>
+      </c>
+      <c r="E9" s="12" t="n">
+        <v>253.8</v>
+      </c>
+      <c r="F9" s="13" t="n">
+        <v>0.5065</v>
       </c>
     </row>
   </sheetData>

</xml_diff>